<commit_message>
Refactor PDF extraction pipeline and add LLM extraction
# Conflicts:
#	extraction-2.py
</commit_message>
<xml_diff>
--- a/pdf_classification.xlsx
+++ b/pdf_classification.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Classification" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classification" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -430,42 +442,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>File Name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Pages</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>PDF Type</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Multi Page</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Text Length</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Image Count</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>OCR Applied</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>OCR Text</t>
         </is>
@@ -501,7 +513,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H2" s="1" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>FDA FORM 3500 — MedWatch Adverse Event Report
 U.S. Department of Health and Human Services | Food and Drug Administration | OMB No. 0910-0291 Expires: 09-30-2027
@@ -593,7 +605,7 @@
           <t>No (native text)</t>
         </is>
       </c>
-      <c r="H3" s="1" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>FDA FORM 3500 — MedWatch Adverse Event Report 
 U.S. Department of Health and Human Services | Food and Drug Administration | OMB No. 0910-0291  Expires: 09-30-2027 
@@ -787,7 +799,7 @@
           <t>No (native text)</t>
         </is>
       </c>
-      <c r="H4" s="1" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>FDA FORM 3500 — MedWatch Adverse Event Report 
 U.S. Department of Health and Human Services | Food and Drug Administration | OMB No. 0910-0291  Expires: 09-30-2027 
@@ -980,7 +992,7 @@
           <t>No (native text)</t>
         </is>
       </c>
-      <c r="H5" s="1" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>FDA FORM 3500 — MedWatch Adverse Event Report 
 U.S. Department of Health and Human Services | Food and Drug Administration | OMB No. 0910-0291  Expires: 09-30-2027 
@@ -1173,7 +1185,7 @@
           <t>No (native text)</t>
         </is>
       </c>
-      <c r="H6" s="1" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>FDA FORM 3500 — MedWatch Adverse Event Report 
 U.S. Department of Health and Human Services | Food and Drug Administration | OMB No. 0910-0291  Expires: 09-30-2027 
@@ -1366,7 +1378,7 @@
           <t>No (native text)</t>
         </is>
       </c>
-      <c r="H7" s="1" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>FDA FORM 3500 — MedWatch Adverse Event Report 
 U.S. Department of Health and Human Services | Food and Drug Administration | OMB No. 0910-0291  Expires: 09-30-2027 
@@ -1559,7 +1571,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H8" s="1" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>FDA FORM 3500 — MedWatch Adverse Event Report
 U.S. Department of Health and Human Services | Food and Drug Administration | OMB No. 0910-0291 Expires: 09-30-2027
@@ -1652,7 +1664,7 @@
           <t>No (native text)</t>
         </is>
       </c>
-      <c r="H9" s="1" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>FDA FORM 3500 — MedWatch Adverse Event Report 
 U.S. Department of Health and Human Services | Food and Drug Administration | OMB No. 0910-0291  Expires: 09-30-2027 
@@ -1845,7 +1857,7 @@
           <t>No (native text)</t>
         </is>
       </c>
-      <c r="H10" s="1" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>FDA FORM 3500 — MedWatch Adverse Event Report 
 U.S. Department of Health and Human Services | Food and Drug Administration | OMB No. 0910-0291  Expires: 09-30-2027 
@@ -2037,7 +2049,7 @@
           <t>No (native text)</t>
         </is>
       </c>
-      <c r="H11" s="1" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>FDA FORM 3500 — MedWatch Adverse Event Report 
 U.S. Department of Health and Human Services | Food and Drug Administration | OMB No. 0910-0291  Expires: 09-30-2027 
@@ -2224,7 +2236,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H12" s="1" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>FDA FORM 3500 — MedWatch Adverse Event Report
 U.S. Department of Health and Human Services | Food and Drug Administration | OMB No. 0910-0291 Expires: 09-30-2027
@@ -2315,7 +2327,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H13" s="1" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>FDA FORM 3500 — MedWatch Adverse Event Report
 U.S. Department of Health and Human Services | Food and Drug Administration | OMB No. 0910-0291 Expires: 09-30-2027
@@ -2406,7 +2418,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H14" s="1" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>FDA FORM 3500 — MedWatch Adverse Event Report
 U.S. Department of Health and Human Services | Food and Drug Administration | OMB No. 0910-0291 Expires: 09-30-2027
@@ -2512,7 +2524,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H15" s="1" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>FDA FORM 3500 — MedWatch Adverse Event Report
 U.S. Department of Health and Human Services | Food and Drug Administration | OMB No. 0910-0291 Expires: 09-30-2027
@@ -2603,7 +2615,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H16" s="1" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>FDA FORM 3500 — MedWatch Adverse Event Report
 U.S. Department of Health and Human Services | Food and Drug Administration | OMB No. 0910-0291 Expires: 09-30-2027
@@ -2694,7 +2706,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H17" s="1" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>FDA FORM 3500 — MedWatch Adverse Event Report
 U.S. Department of Health and Human Services | Food and Drug Administration | OMB No. 0910-0291 Expires: 09-30-2027
@@ -2786,7 +2798,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H18" s="1" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>FDA FORM 3500 — MedWatch Adverse Event Report
 U.S. Department of Health and Human Services | Food and Drug Administration | OMB No. 0910-0291 Expires: 09-30-2027
@@ -2878,7 +2890,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H19" s="1" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>FDA FORM 3500 — MedWatch Adverse Event Report
 U.S. Department of Health and Human Services | Food and Drug Administration | OMB No. 0910-0291 Expires: 09-30-2027
@@ -2970,7 +2982,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H20" s="1" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr"/>
     </row>
     <row r="21" ht="300" customHeight="1">
       <c r="A21" t="inlineStr">
@@ -3002,7 +3014,7 @@
           <t>No (native text)</t>
         </is>
       </c>
-      <c r="H21" s="1" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>Welcome 
 app.py 
@@ -3083,7 +3095,7 @@
           <t>No (native text)</t>
         </is>
       </c>
-      <c r="H22" s="1" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>FDA FORM 3500 — MedWatch Adverse Event Report 
 U.S. Department of Health and Human Services | Food and Drug Administration | OMB No. 0910-0291  Expires: 09-30-2027 
@@ -3276,7 +3288,7 @@
           <t>No (native text)</t>
         </is>
       </c>
-      <c r="H23" s="1" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>FDA FORM 3500 — MedWatch Adverse Event Report 
 U.S. Department of Health and Human Services | Food and Drug Administration | OMB No. 0910-0291  Expires: 09-30-2027 

</xml_diff>